<commit_message>
LyreViz : longueur exacte des faisceaux arrêtés par le sol (le bout des taches vues en rasant n'est plus coupé net), vue d'essai --demo 4 (pont de scène en rasant), historique et documentation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lyre-viz/historique_perf.xlsx
+++ b/lyre-viz/historique_perf.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O224"/>
+  <dimension ref="A1:O240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -13430,6 +13430,938 @@
         </is>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="n">
+        <v>8.535</v>
+      </c>
+      <c r="H225" s="4">
+        <f>IF(G225&gt;0,1000/G225,"")</f>
+        <v/>
+      </c>
+      <c r="I225" s="3" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="J225" s="3" t="n">
+        <v>6.985</v>
+      </c>
+      <c r="K225" s="3" t="n">
+        <v>1.621</v>
+      </c>
+      <c r="L225" s="3" t="n">
+        <v>1.946</v>
+      </c>
+      <c r="M225" s="3" t="n"/>
+      <c r="N225" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O225" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>defaut / scene</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="n">
+        <v>8.025</v>
+      </c>
+      <c r="H226" s="4">
+        <f>IF(G226&gt;0,1000/G226,"")</f>
+        <v/>
+      </c>
+      <c r="I226" s="3" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="J226" s="3" t="n">
+        <v>6.835</v>
+      </c>
+      <c r="K226" s="3" t="n">
+        <v>1.601</v>
+      </c>
+      <c r="L226" s="3" t="n">
+        <v>1.861</v>
+      </c>
+      <c r="M226" s="3" t="n"/>
+      <c r="N226" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O226" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>defaut / sous les trusses</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="n">
+        <v>7.745</v>
+      </c>
+      <c r="H227" s="4">
+        <f>IF(G227&gt;0,1000/G227,"")</f>
+        <v/>
+      </c>
+      <c r="I227" s="3" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="J227" s="3" t="n">
+        <v>5.625</v>
+      </c>
+      <c r="K227" s="3" t="n">
+        <v>1.106</v>
+      </c>
+      <c r="L227" s="3" t="n">
+        <v>1.542</v>
+      </c>
+      <c r="M227" s="3" t="n"/>
+      <c r="N227" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O227" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G228" s="3" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="H228" s="4">
+        <f>IF(G228&gt;0,1000/G228,"")</f>
+        <v/>
+      </c>
+      <c r="I228" s="3" t="n">
+        <v>18.445</v>
+      </c>
+      <c r="J228" s="3" t="n">
+        <v>18.495</v>
+      </c>
+      <c r="K228" s="3" t="n">
+        <v>6.735</v>
+      </c>
+      <c r="L228" s="3" t="n">
+        <v>6.984</v>
+      </c>
+      <c r="M228" s="3" t="n"/>
+      <c r="N228" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O228" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / scene</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="n">
+        <v>18.335</v>
+      </c>
+      <c r="H229" s="4">
+        <f>IF(G229&gt;0,1000/G229,"")</f>
+        <v/>
+      </c>
+      <c r="I229" s="3" t="n">
+        <v>17.475</v>
+      </c>
+      <c r="J229" s="3" t="n">
+        <v>17.125</v>
+      </c>
+      <c r="K229" s="3" t="n">
+        <v>6.085</v>
+      </c>
+      <c r="L229" s="3" t="n">
+        <v>6.376</v>
+      </c>
+      <c r="M229" s="3" t="n"/>
+      <c r="N229" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O229" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / sous les trusses</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="n">
+        <v>13.695</v>
+      </c>
+      <c r="H230" s="4">
+        <f>IF(G230&gt;0,1000/G230,"")</f>
+        <v/>
+      </c>
+      <c r="I230" s="3" t="n">
+        <v>13.005</v>
+      </c>
+      <c r="J230" s="3" t="n">
+        <v>13.095</v>
+      </c>
+      <c r="K230" s="3" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="L230" s="3" t="n">
+        <v>4.087</v>
+      </c>
+      <c r="M230" s="3" t="n"/>
+      <c r="N230" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O230" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G231" s="3" t="n">
+        <v>11.775</v>
+      </c>
+      <c r="H231" s="4">
+        <f>IF(G231&gt;0,1000/G231,"")</f>
+        <v/>
+      </c>
+      <c r="I231" s="3" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="J231" s="3" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="K231" s="3" t="n">
+        <v>3.396</v>
+      </c>
+      <c r="L231" s="3" t="n">
+        <v>4.079</v>
+      </c>
+      <c r="M231" s="3" t="n"/>
+      <c r="N231" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O231" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / scene</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="n">
+        <v>11.81</v>
+      </c>
+      <c r="H232" s="4">
+        <f>IF(G232&gt;0,1000/G232,"")</f>
+        <v/>
+      </c>
+      <c r="I232" s="3" t="n">
+        <v>10.975</v>
+      </c>
+      <c r="J232" s="3" t="n">
+        <v>10.725</v>
+      </c>
+      <c r="K232" s="3" t="n">
+        <v>2.983</v>
+      </c>
+      <c r="L232" s="3" t="n">
+        <v>4.072</v>
+      </c>
+      <c r="M232" s="3" t="n"/>
+      <c r="N232" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O232" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / sous les trusses</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="H233" s="4">
+        <f>IF(G233&gt;0,1000/G233,"")</f>
+        <v/>
+      </c>
+      <c r="I233" s="3" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="J233" s="3" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="K233" s="3" t="n">
+        <v>1.511</v>
+      </c>
+      <c r="L233" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M233" s="3" t="n"/>
+      <c r="N233" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O233" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>sans rebonds (GI)</t>
+        </is>
+      </c>
+      <c r="G234" s="3" t="n">
+        <v>7.815</v>
+      </c>
+      <c r="H234" s="4">
+        <f>IF(G234&gt;0,1000/G234,"")</f>
+        <v/>
+      </c>
+      <c r="I234" s="3" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="J234" s="3" t="n">
+        <v>5.995</v>
+      </c>
+      <c r="K234" s="3" t="n">
+        <v>1.422</v>
+      </c>
+      <c r="L234" s="3" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="M234" s="3" t="n"/>
+      <c r="N234" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O234" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>sans fumee volumetrique</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="n">
+        <v>5.155</v>
+      </c>
+      <c r="H235" s="4">
+        <f>IF(G235&gt;0,1000/G235,"")</f>
+        <v/>
+      </c>
+      <c r="I235" s="3" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="J235" s="3" t="n">
+        <v>2.985</v>
+      </c>
+      <c r="K235" s="3" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="L235" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M235" s="3" t="n"/>
+      <c r="N235" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O235" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>sans taches sur surfaces</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="H236" s="4">
+        <f>IF(G236&gt;0,1000/G236,"")</f>
+        <v/>
+      </c>
+      <c r="I236" s="3" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="J236" s="3" t="n">
+        <v>5.905</v>
+      </c>
+      <c r="K236" s="3" t="n">
+        <v>0.699</v>
+      </c>
+      <c r="L236" s="3" t="n">
+        <v>1.922</v>
+      </c>
+      <c r="M236" s="3" t="n"/>
+      <c r="N236" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O236" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>sans reflets</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="H237" s="4">
+        <f>IF(G237&gt;0,1000/G237,"")</f>
+        <v/>
+      </c>
+      <c r="I237" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="J237" s="3" t="n">
+        <v>6.835</v>
+      </c>
+      <c r="K237" s="3" t="n">
+        <v>1.619</v>
+      </c>
+      <c r="L237" s="3" t="n">
+        <v>1.971</v>
+      </c>
+      <c r="M237" s="3" t="n"/>
+      <c r="N237" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O237" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>sans bloom</t>
+        </is>
+      </c>
+      <c r="G238" s="3" t="n">
+        <v>7.785</v>
+      </c>
+      <c r="H238" s="4">
+        <f>IF(G238&gt;0,1000/G238,"")</f>
+        <v/>
+      </c>
+      <c r="I238" s="3" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="J238" s="3" t="n">
+        <v>6.155</v>
+      </c>
+      <c r="K238" s="3" t="n">
+        <v>1.607</v>
+      </c>
+      <c r="L238" s="3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="M238" s="3" t="n"/>
+      <c r="N238" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O238" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>sol mouille / public</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="n">
+        <v>10.135</v>
+      </c>
+      <c r="H239" s="4">
+        <f>IF(G239&gt;0,1000/G239,"")</f>
+        <v/>
+      </c>
+      <c r="I239" s="3" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="J239" s="3" t="n">
+        <v>9.215</v>
+      </c>
+      <c r="K239" s="3" t="n">
+        <v>1.773</v>
+      </c>
+      <c r="L239" s="3" t="n">
+        <v>2.058</v>
+      </c>
+      <c r="M239" s="3" t="n">
+        <v>1.046</v>
+      </c>
+      <c r="N239" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O239" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 21:58</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>403cbd3 +modifs</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (--fast)</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>sol mouille + gobo + prisme 8 / scene</t>
+        </is>
+      </c>
+      <c r="G240" s="3" t="n">
+        <v>22.755</v>
+      </c>
+      <c r="H240" s="4">
+        <f>IF(G240&gt;0,1000/G240,"")</f>
+        <v/>
+      </c>
+      <c r="I240" s="3" t="n">
+        <v>22.225</v>
+      </c>
+      <c r="J240" s="3" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="K240" s="3" t="n">
+        <v>5.387</v>
+      </c>
+      <c r="L240" s="3" t="n">
+        <v>6.576</v>
+      </c>
+      <c r="M240" s="3" t="n">
+        <v>3.983</v>
+      </c>
+      <c r="N240" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O240" s="2" t="inlineStr">
+        <is>
+          <t>longueur2_B0, longueur2_B1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13441,7 +14373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13460,6 +14392,7 @@
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13550,6 +14483,11 @@
           <t>7e4. Essai v4 : cache recalcule s'il change (RGBA16F), chroma=1</t>
         </is>
       </c>
+      <c r="Q2" s="1" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -13617,6 +14555,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -13684,6 +14626,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -13751,6 +14697,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -13818,6 +14768,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -13885,6 +14839,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -13952,6 +14910,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -14019,6 +14981,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -14086,6 +15052,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -14153,6 +15123,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -14220,6 +15194,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -14287,6 +15265,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -14354,6 +15336,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -14421,6 +15407,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -14488,6 +15478,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -14555,6 +15549,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -14622,6 +15620,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,P$2),"")</f>
         <v/>
       </c>
+      <c r="Q18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,Q$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -14711,6 +15713,11 @@
           <t>7e4. Essai v4 : cache recalcule s'il change (RGBA16F), chroma=1</t>
         </is>
       </c>
+      <c r="Q21" s="1" t="inlineStr">
+        <is>
+          <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -14778,6 +15785,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -14845,6 +15856,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -14912,6 +15927,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -14979,6 +15998,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -15046,6 +16069,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -15113,6 +16140,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -15180,6 +16211,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -15247,6 +16282,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -15314,6 +16353,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -15381,6 +16424,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -15448,6 +16495,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -15515,6 +16566,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -15582,6 +16637,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -15649,6 +16708,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -15716,6 +16779,10 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,P$21),"")</f>
         <v/>
       </c>
+      <c r="Q36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -15781,6 +16848,10 @@
       </c>
       <c r="P37" s="3">
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,P$21),"")</f>
+        <v/>
+      </c>
+      <c r="Q37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
LyreViz : eau au sol refaite (creux du béton remplis d'abord, puis flaques de plus en plus grandes, reflet net seulement dans l'eau, variantes sèche et mouillée de la passe des surfaces) et reflet calculé seulement dans l'eau (masque par blocs), vue d'essai --demo 5, historique et documentation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lyre-viz/historique_perf.xlsx
+++ b/lyre-viz/historique_perf.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O240"/>
+  <dimension ref="A1:O277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -14362,6 +14362,2198 @@
         </is>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G241" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H241" s="4">
+        <f>IF(G241&gt;0,1000/G241,"")</f>
+        <v/>
+      </c>
+      <c r="I241" s="3" t="n">
+        <v>7.435</v>
+      </c>
+      <c r="J241" s="3" t="n">
+        <v>6.73</v>
+      </c>
+      <c r="K241" s="3" t="n">
+        <v>1.631</v>
+      </c>
+      <c r="L241" s="3" t="n">
+        <v>1.988</v>
+      </c>
+      <c r="M241" s="3" t="n"/>
+      <c r="N241" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O241" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>defaut / scene</t>
+        </is>
+      </c>
+      <c r="G242" s="3" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="H242" s="4">
+        <f>IF(G242&gt;0,1000/G242,"")</f>
+        <v/>
+      </c>
+      <c r="I242" s="3" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="J242" s="3" t="n">
+        <v>6.865</v>
+      </c>
+      <c r="K242" s="3" t="n">
+        <v>1.579</v>
+      </c>
+      <c r="L242" s="3" t="n">
+        <v>1.954</v>
+      </c>
+      <c r="M242" s="3" t="n"/>
+      <c r="N242" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O242" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>defaut / sous les trusses</t>
+        </is>
+      </c>
+      <c r="G243" s="3" t="n">
+        <v>8.074999999999999</v>
+      </c>
+      <c r="H243" s="4">
+        <f>IF(G243&gt;0,1000/G243,"")</f>
+        <v/>
+      </c>
+      <c r="I243" s="3" t="n">
+        <v>6.475</v>
+      </c>
+      <c r="J243" s="3" t="n">
+        <v>6.125</v>
+      </c>
+      <c r="K243" s="3" t="n">
+        <v>1.131</v>
+      </c>
+      <c r="L243" s="3" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="M243" s="3" t="n"/>
+      <c r="N243" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O243" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G244" s="3" t="n">
+        <v>20.835</v>
+      </c>
+      <c r="H244" s="4">
+        <f>IF(G244&gt;0,1000/G244,"")</f>
+        <v/>
+      </c>
+      <c r="I244" s="3" t="n">
+        <v>19.575</v>
+      </c>
+      <c r="J244" s="3" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="K244" s="3" t="n">
+        <v>7.428</v>
+      </c>
+      <c r="L244" s="3" t="n">
+        <v>6.918</v>
+      </c>
+      <c r="M244" s="3" t="n"/>
+      <c r="N244" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O244" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / scene</t>
+        </is>
+      </c>
+      <c r="G245" s="3" t="n">
+        <v>19.185</v>
+      </c>
+      <c r="H245" s="4">
+        <f>IF(G245&gt;0,1000/G245,"")</f>
+        <v/>
+      </c>
+      <c r="I245" s="3" t="n">
+        <v>18.005</v>
+      </c>
+      <c r="J245" s="3" t="n">
+        <v>17.835</v>
+      </c>
+      <c r="K245" s="3" t="n">
+        <v>5.706</v>
+      </c>
+      <c r="L245" s="3" t="n">
+        <v>6.345</v>
+      </c>
+      <c r="M245" s="3" t="n"/>
+      <c r="N245" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O245" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / sous les trusses</t>
+        </is>
+      </c>
+      <c r="G246" s="3" t="n">
+        <v>14.61</v>
+      </c>
+      <c r="H246" s="4">
+        <f>IF(G246&gt;0,1000/G246,"")</f>
+        <v/>
+      </c>
+      <c r="I246" s="3" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="J246" s="3" t="n">
+        <v>13.97</v>
+      </c>
+      <c r="K246" s="3" t="n">
+        <v>3.371</v>
+      </c>
+      <c r="L246" s="3" t="n">
+        <v>3.962</v>
+      </c>
+      <c r="M246" s="3" t="n"/>
+      <c r="N246" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O246" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G247" s="3" t="n">
+        <v>12.575</v>
+      </c>
+      <c r="H247" s="4">
+        <f>IF(G247&gt;0,1000/G247,"")</f>
+        <v/>
+      </c>
+      <c r="I247" s="3" t="n">
+        <v>11.245</v>
+      </c>
+      <c r="J247" s="3" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="K247" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L247" s="3" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="M247" s="3" t="n"/>
+      <c r="N247" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O247" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / scene</t>
+        </is>
+      </c>
+      <c r="G248" s="3" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H248" s="4">
+        <f>IF(G248&gt;0,1000/G248,"")</f>
+        <v/>
+      </c>
+      <c r="I248" s="3" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="J248" s="3" t="n">
+        <v>10.115</v>
+      </c>
+      <c r="K248" s="3" t="n">
+        <v>2.965</v>
+      </c>
+      <c r="L248" s="3" t="n">
+        <v>4.127</v>
+      </c>
+      <c r="M248" s="3" t="n"/>
+      <c r="N248" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O248" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / sous les trusses</t>
+        </is>
+      </c>
+      <c r="G249" s="3" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="H249" s="4">
+        <f>IF(G249&gt;0,1000/G249,"")</f>
+        <v/>
+      </c>
+      <c r="I249" s="3" t="n">
+        <v>8.27</v>
+      </c>
+      <c r="J249" s="3" t="n">
+        <v>7.685</v>
+      </c>
+      <c r="K249" s="3" t="n">
+        <v>1.527</v>
+      </c>
+      <c r="L249" s="3" t="n">
+        <v>3.239</v>
+      </c>
+      <c r="M249" s="3" t="n"/>
+      <c r="N249" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O249" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>sans rebonds (GI)</t>
+        </is>
+      </c>
+      <c r="G250" s="3" t="n">
+        <v>7.805</v>
+      </c>
+      <c r="H250" s="4">
+        <f>IF(G250&gt;0,1000/G250,"")</f>
+        <v/>
+      </c>
+      <c r="I250" s="3" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="J250" s="3" t="n">
+        <v>5.915</v>
+      </c>
+      <c r="K250" s="3" t="n">
+        <v>1.406</v>
+      </c>
+      <c r="L250" s="3" t="n">
+        <v>1.526</v>
+      </c>
+      <c r="M250" s="3" t="n"/>
+      <c r="N250" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O250" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>sans fumee volumetrique</t>
+        </is>
+      </c>
+      <c r="G251" s="3" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="H251" s="4">
+        <f>IF(G251&gt;0,1000/G251,"")</f>
+        <v/>
+      </c>
+      <c r="I251" s="3" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="J251" s="3" t="n">
+        <v>3.215</v>
+      </c>
+      <c r="K251" s="3" t="n">
+        <v>1.663</v>
+      </c>
+      <c r="L251" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M251" s="3" t="n"/>
+      <c r="N251" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O251" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>sans taches sur surfaces</t>
+        </is>
+      </c>
+      <c r="G252" s="3" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="H252" s="4">
+        <f>IF(G252&gt;0,1000/G252,"")</f>
+        <v/>
+      </c>
+      <c r="I252" s="3" t="n">
+        <v>6.585</v>
+      </c>
+      <c r="J252" s="3" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="K252" s="3" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="L252" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M252" s="3" t="n"/>
+      <c r="N252" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O252" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>sans reflets</t>
+        </is>
+      </c>
+      <c r="G253" s="3" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="H253" s="4">
+        <f>IF(G253&gt;0,1000/G253,"")</f>
+        <v/>
+      </c>
+      <c r="I253" s="3" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="J253" s="3" t="n">
+        <v>7.625</v>
+      </c>
+      <c r="K253" s="3" t="n">
+        <v>1.667</v>
+      </c>
+      <c r="L253" s="3" t="n">
+        <v>2.005</v>
+      </c>
+      <c r="M253" s="3" t="n"/>
+      <c r="N253" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O253" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>sans bloom</t>
+        </is>
+      </c>
+      <c r="G254" s="3" t="n">
+        <v>8.025</v>
+      </c>
+      <c r="H254" s="4">
+        <f>IF(G254&gt;0,1000/G254,"")</f>
+        <v/>
+      </c>
+      <c r="I254" s="3" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="J254" s="3" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="K254" s="3" t="n">
+        <v>1.629</v>
+      </c>
+      <c r="L254" s="3" t="n">
+        <v>1.977</v>
+      </c>
+      <c r="M254" s="3" t="n"/>
+      <c r="N254" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O254" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>sol mouille / public</t>
+        </is>
+      </c>
+      <c r="G255" s="3" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="H255" s="4">
+        <f>IF(G255&gt;0,1000/G255,"")</f>
+        <v/>
+      </c>
+      <c r="I255" s="3" t="n">
+        <v>9.515000000000001</v>
+      </c>
+      <c r="J255" s="3" t="n">
+        <v>9.205</v>
+      </c>
+      <c r="K255" s="3" t="n">
+        <v>2.049</v>
+      </c>
+      <c r="L255" s="3" t="n">
+        <v>2.061</v>
+      </c>
+      <c r="M255" s="3" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="N255" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O255" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide (cas 15-16 : eau 0,8)</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>sol mouille + gobo + prisme 8 / scene</t>
+        </is>
+      </c>
+      <c r="G256" s="3" t="n">
+        <v>24.49</v>
+      </c>
+      <c r="H256" s="4">
+        <f>IF(G256&gt;0,1000/G256,"")</f>
+        <v/>
+      </c>
+      <c r="I256" s="3" t="n">
+        <v>23.765</v>
+      </c>
+      <c r="J256" s="3" t="n">
+        <v>23.545</v>
+      </c>
+      <c r="K256" s="3" t="n">
+        <v>6.349</v>
+      </c>
+      <c r="L256" s="3" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="M256" s="3" t="n">
+        <v>4.784</v>
+      </c>
+      <c r="N256" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O256" s="2" t="inlineStr">
+        <is>
+          <t>eau2_B0, eau2_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>9b. Eau au sol a 10 %</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G257" s="3" t="n">
+        <v>10.335</v>
+      </c>
+      <c r="H257" s="4">
+        <f>IF(G257&gt;0,1000/G257,"")</f>
+        <v/>
+      </c>
+      <c r="I257" s="3" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="J257" s="3" t="n">
+        <v>9.205</v>
+      </c>
+      <c r="K257" s="3" t="n">
+        <v>1.978</v>
+      </c>
+      <c r="L257" s="3" t="n">
+        <v>1.968</v>
+      </c>
+      <c r="M257" s="3" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="N257" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O257" s="2" t="inlineStr">
+        <is>
+          <t>eau2_10_B0, eau2_10_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>9b. Eau au sol a 10 %</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G258" s="3" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="H258" s="4">
+        <f>IF(G258&gt;0,1000/G258,"")</f>
+        <v/>
+      </c>
+      <c r="I258" s="3" t="n">
+        <v>25.65</v>
+      </c>
+      <c r="J258" s="3" t="n">
+        <v>25.275</v>
+      </c>
+      <c r="K258" s="3" t="n">
+        <v>7.163</v>
+      </c>
+      <c r="L258" s="3" t="n">
+        <v>6.729</v>
+      </c>
+      <c r="M258" s="3" t="n">
+        <v>5.549</v>
+      </c>
+      <c r="N258" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O258" s="2" t="inlineStr">
+        <is>
+          <t>eau2_10_B0, eau2_10_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>9b. Eau au sol a 10 %</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G259" s="3" t="n">
+        <v>23.265</v>
+      </c>
+      <c r="H259" s="4">
+        <f>IF(G259&gt;0,1000/G259,"")</f>
+        <v/>
+      </c>
+      <c r="I259" s="3" t="n">
+        <v>21.995</v>
+      </c>
+      <c r="J259" s="3" t="n">
+        <v>21.65</v>
+      </c>
+      <c r="K259" s="3" t="n">
+        <v>3.192</v>
+      </c>
+      <c r="L259" s="3" t="n">
+        <v>3.938</v>
+      </c>
+      <c r="M259" s="3" t="n">
+        <v>10.626</v>
+      </c>
+      <c r="N259" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O259" s="2" t="inlineStr">
+        <is>
+          <t>eau2_10_B0, eau2_10_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>9e. Essai : creux en trilineaire (abandonne)</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G260" s="3" t="n">
+        <v>10.443</v>
+      </c>
+      <c r="H260" s="4">
+        <f>IF(G260&gt;0,1000/G260,"")</f>
+        <v/>
+      </c>
+      <c r="I260" s="3" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="J260" s="3" t="n">
+        <v>9.167</v>
+      </c>
+      <c r="K260" s="3" t="n">
+        <v>1.981</v>
+      </c>
+      <c r="L260" s="3" t="n">
+        <v>1.977</v>
+      </c>
+      <c r="M260" s="3" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="N260" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O260" s="2" t="inlineStr">
+        <is>
+          <t>eau3_B0, eau3_B1, eau3_B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>9e. Essai : creux en trilineaire (abandonne)</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G261" s="3" t="n">
+        <v>25.493</v>
+      </c>
+      <c r="H261" s="4">
+        <f>IF(G261&gt;0,1000/G261,"")</f>
+        <v/>
+      </c>
+      <c r="I261" s="3" t="n">
+        <v>24.817</v>
+      </c>
+      <c r="J261" s="3" t="n">
+        <v>24.72</v>
+      </c>
+      <c r="K261" s="3" t="n">
+        <v>7.241</v>
+      </c>
+      <c r="L261" s="3" t="n">
+        <v>6.729</v>
+      </c>
+      <c r="M261" s="3" t="n">
+        <v>5.336</v>
+      </c>
+      <c r="N261" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O261" s="2" t="inlineStr">
+        <is>
+          <t>eau3_B0, eau3_B1, eau3_B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:37</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>9e. Essai : creux en trilineaire (abandonne)</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G262" s="3" t="n">
+        <v>22.373</v>
+      </c>
+      <c r="H262" s="4">
+        <f>IF(G262&gt;0,1000/G262,"")</f>
+        <v/>
+      </c>
+      <c r="I262" s="3" t="n">
+        <v>21.39</v>
+      </c>
+      <c r="J262" s="3" t="n">
+        <v>21.117</v>
+      </c>
+      <c r="K262" s="3" t="n">
+        <v>3.085</v>
+      </c>
+      <c r="L262" s="3" t="n">
+        <v>3.904</v>
+      </c>
+      <c r="M262" s="3" t="n">
+        <v>10.149</v>
+      </c>
+      <c r="N262" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O262" s="2" t="inlineStr">
+        <is>
+          <t>eau3_B0, eau3_B1, eau3_B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>10a. Reflet seulement dans l'eau (masque par blocs), eau 0,1</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G263" s="3" t="n">
+        <v>10.435</v>
+      </c>
+      <c r="H263" s="4">
+        <f>IF(G263&gt;0,1000/G263,"")</f>
+        <v/>
+      </c>
+      <c r="I263" s="3" t="n">
+        <v>9.335000000000001</v>
+      </c>
+      <c r="J263" s="3" t="n">
+        <v>9.140000000000001</v>
+      </c>
+      <c r="K263" s="3" t="n">
+        <v>1.974</v>
+      </c>
+      <c r="L263" s="3" t="n">
+        <v>2.058</v>
+      </c>
+      <c r="M263" s="3" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="N263" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O263" s="2" t="inlineStr">
+        <is>
+          <t>masque_w01_B0, masque_w01_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>10a. Reflet seulement dans l'eau (masque par blocs), eau 0,1</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G264" s="3" t="n">
+        <v>24.45</v>
+      </c>
+      <c r="H264" s="4">
+        <f>IF(G264&gt;0,1000/G264,"")</f>
+        <v/>
+      </c>
+      <c r="I264" s="3" t="n">
+        <v>23.745</v>
+      </c>
+      <c r="J264" s="3" t="n">
+        <v>23.73</v>
+      </c>
+      <c r="K264" s="3" t="n">
+        <v>7.047</v>
+      </c>
+      <c r="L264" s="3" t="n">
+        <v>6.708</v>
+      </c>
+      <c r="M264" s="3" t="n">
+        <v>4.266</v>
+      </c>
+      <c r="N264" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O264" s="2" t="inlineStr">
+        <is>
+          <t>masque_w01_B0, masque_w01_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>10a. Reflet seulement dans l'eau (masque par blocs), eau 0,1</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G265" s="3" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="H265" s="4">
+        <f>IF(G265&gt;0,1000/G265,"")</f>
+        <v/>
+      </c>
+      <c r="I265" s="3" t="n">
+        <v>17.035</v>
+      </c>
+      <c r="J265" s="3" t="n">
+        <v>17.245</v>
+      </c>
+      <c r="K265" s="3" t="n">
+        <v>3.214</v>
+      </c>
+      <c r="L265" s="3" t="n">
+        <v>4.069</v>
+      </c>
+      <c r="M265" s="3" t="n">
+        <v>5.796</v>
+      </c>
+      <c r="N265" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O265" s="2" t="inlineStr">
+        <is>
+          <t>masque_w01_B0, masque_w01_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>10b. Reflet seulement dans l'eau, eau 0,3</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G266" s="3" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="H266" s="4">
+        <f>IF(G266&gt;0,1000/G266,"")</f>
+        <v/>
+      </c>
+      <c r="I266" s="3" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="J266" s="3" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="K266" s="3" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="L266" s="3" t="n">
+        <v>2.033</v>
+      </c>
+      <c r="M266" s="3" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="N266" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O266" s="2" t="inlineStr">
+        <is>
+          <t>masque30d_B0, masque30d_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>10b. Reflet seulement dans l'eau, eau 0,3</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G267" s="3" t="n">
+        <v>24.965</v>
+      </c>
+      <c r="H267" s="4">
+        <f>IF(G267&gt;0,1000/G267,"")</f>
+        <v/>
+      </c>
+      <c r="I267" s="3" t="n">
+        <v>24.46</v>
+      </c>
+      <c r="J267" s="3" t="n">
+        <v>24.39</v>
+      </c>
+      <c r="K267" s="3" t="n">
+        <v>7.035</v>
+      </c>
+      <c r="L267" s="3" t="n">
+        <v>6.774</v>
+      </c>
+      <c r="M267" s="3" t="n">
+        <v>5.058</v>
+      </c>
+      <c r="N267" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O267" s="2" t="inlineStr">
+        <is>
+          <t>masque30d_B0, masque30d_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>10b. Reflet seulement dans l'eau, eau 0,3</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G268" s="3" t="n">
+        <v>20.31</v>
+      </c>
+      <c r="H268" s="4">
+        <f>IF(G268&gt;0,1000/G268,"")</f>
+        <v/>
+      </c>
+      <c r="I268" s="3" t="n">
+        <v>19.29</v>
+      </c>
+      <c r="J268" s="3" t="n">
+        <v>19.255</v>
+      </c>
+      <c r="K268" s="3" t="n">
+        <v>3.122</v>
+      </c>
+      <c r="L268" s="3" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="M268" s="3" t="n">
+        <v>8.183</v>
+      </c>
+      <c r="N268" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O268" s="2" t="inlineStr">
+        <is>
+          <t>masque30d_B0, masque30d_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>10c. Reflet seulement dans l'eau, eau 1</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G269" s="3" t="n">
+        <v>10.545</v>
+      </c>
+      <c r="H269" s="4">
+        <f>IF(G269&gt;0,1000/G269,"")</f>
+        <v/>
+      </c>
+      <c r="I269" s="3" t="n">
+        <v>9.395</v>
+      </c>
+      <c r="J269" s="3" t="n">
+        <v>8.895</v>
+      </c>
+      <c r="K269" s="3" t="n">
+        <v>1.987</v>
+      </c>
+      <c r="L269" s="3" t="n">
+        <v>2.047</v>
+      </c>
+      <c r="M269" s="3" t="n">
+        <v>1.036</v>
+      </c>
+      <c r="N269" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O269" s="2" t="inlineStr">
+        <is>
+          <t>masque_w1_B0, masque_w1_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>10c. Reflet seulement dans l'eau, eau 1</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G270" s="3" t="n">
+        <v>24.72</v>
+      </c>
+      <c r="H270" s="4">
+        <f>IF(G270&gt;0,1000/G270,"")</f>
+        <v/>
+      </c>
+      <c r="I270" s="3" t="n">
+        <v>24.025</v>
+      </c>
+      <c r="J270" s="3" t="n">
+        <v>23.955</v>
+      </c>
+      <c r="K270" s="3" t="n">
+        <v>6.742</v>
+      </c>
+      <c r="L270" s="3" t="n">
+        <v>6.862</v>
+      </c>
+      <c r="M270" s="3" t="n">
+        <v>4.739</v>
+      </c>
+      <c r="N270" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O270" s="2" t="inlineStr">
+        <is>
+          <t>masque_w1_B0, masque_w1_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>10c. Reflet seulement dans l'eau, eau 1</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=1, 3 cas</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G271" s="3" t="n">
+        <v>22.225</v>
+      </c>
+      <c r="H271" s="4">
+        <f>IF(G271&gt;0,1000/G271,"")</f>
+        <v/>
+      </c>
+      <c r="I271" s="3" t="n">
+        <v>21.025</v>
+      </c>
+      <c r="J271" s="3" t="n">
+        <v>20.725</v>
+      </c>
+      <c r="K271" s="3" t="n">
+        <v>3.311</v>
+      </c>
+      <c r="L271" s="3" t="n">
+        <v>4.068</v>
+      </c>
+      <c r="M271" s="3" t="n">
+        <v>9.781000000000001</v>
+      </c>
+      <c r="N271" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O271" s="2" t="inlineStr">
+        <is>
+          <t>masque_w1_B0, masque_w1_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>10e1. Essai masque : 1 point par pixel du miroir (creux manques)</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G272" s="3" t="n">
+        <v>10.185</v>
+      </c>
+      <c r="H272" s="4">
+        <f>IF(G272&gt;0,1000/G272,"")</f>
+        <v/>
+      </c>
+      <c r="I272" s="3" t="n">
+        <v>8.275</v>
+      </c>
+      <c r="J272" s="3" t="n">
+        <v>7.925</v>
+      </c>
+      <c r="K272" s="3" t="n">
+        <v>1.976</v>
+      </c>
+      <c r="L272" s="3" t="n">
+        <v>2.026</v>
+      </c>
+      <c r="M272" s="3" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="N272" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O272" s="2" t="inlineStr">
+        <is>
+          <t>masque30_B0, masque30_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>10e1. Essai masque : 1 point par pixel du miroir (creux manques)</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G273" s="3" t="n">
+        <v>22.795</v>
+      </c>
+      <c r="H273" s="4">
+        <f>IF(G273&gt;0,1000/G273,"")</f>
+        <v/>
+      </c>
+      <c r="I273" s="3" t="n">
+        <v>22.29</v>
+      </c>
+      <c r="J273" s="3" t="n">
+        <v>22.145</v>
+      </c>
+      <c r="K273" s="3" t="n">
+        <v>6.997</v>
+      </c>
+      <c r="L273" s="3" t="n">
+        <v>6.96</v>
+      </c>
+      <c r="M273" s="3" t="n">
+        <v>3.037</v>
+      </c>
+      <c r="N273" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O273" s="2" t="inlineStr">
+        <is>
+          <t>masque30_B0, masque30_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>10e1. Essai masque : 1 point par pixel du miroir (creux manques)</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G274" s="3" t="n">
+        <v>17.785</v>
+      </c>
+      <c r="H274" s="4">
+        <f>IF(G274&gt;0,1000/G274,"")</f>
+        <v/>
+      </c>
+      <c r="I274" s="3" t="n">
+        <v>17.11</v>
+      </c>
+      <c r="J274" s="3" t="n">
+        <v>16.58</v>
+      </c>
+      <c r="K274" s="3" t="n">
+        <v>3.274</v>
+      </c>
+      <c r="L274" s="3" t="n">
+        <v>4.053</v>
+      </c>
+      <c r="M274" s="3" t="n">
+        <v>6.131</v>
+      </c>
+      <c r="N274" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O274" s="2" t="inlineStr">
+        <is>
+          <t>masque30_B0, masque30_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>10e3. Essai masque : faisceaux seulement dans les flaques (pores plus sombres)</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>defaut / public</t>
+        </is>
+      </c>
+      <c r="G275" s="3" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="H275" s="4">
+        <f>IF(G275&gt;0,1000/G275,"")</f>
+        <v/>
+      </c>
+      <c r="I275" s="3" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="J275" s="3" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="K275" s="3" t="n">
+        <v>1.969</v>
+      </c>
+      <c r="L275" s="3" t="n">
+        <v>2.051</v>
+      </c>
+      <c r="M275" s="3" t="n">
+        <v>0.783</v>
+      </c>
+      <c r="N275" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="O275" s="2" t="inlineStr">
+        <is>
+          <t>masque30c_B0, masque30c_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>10e3. Essai masque : faisceaux seulement dans les flaques (pores plus sombres)</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>gobo + prisme 8 + zoom 25 / public</t>
+        </is>
+      </c>
+      <c r="G276" s="3" t="n">
+        <v>24.63</v>
+      </c>
+      <c r="H276" s="4">
+        <f>IF(G276&gt;0,1000/G276,"")</f>
+        <v/>
+      </c>
+      <c r="I276" s="3" t="n">
+        <v>24.06</v>
+      </c>
+      <c r="J276" s="3" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="K276" s="3" t="n">
+        <v>7.072</v>
+      </c>
+      <c r="L276" s="3" t="n">
+        <v>6.812</v>
+      </c>
+      <c r="M276" s="3" t="n">
+        <v>4.506</v>
+      </c>
+      <c r="N276" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="O276" s="2" t="inlineStr">
+        <is>
+          <t>masque30c_B0, masque30c_B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 22:55</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>f23a476+modifs</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>10e3. Essai masque : faisceaux seulement dans les flaques (pores plus sombres)</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>adaptive=0, immobile, banc rapide, wet=0.3, 3 cas</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>zoom 45 + frost 0.6 / public</t>
+        </is>
+      </c>
+      <c r="G277" s="3" t="n">
+        <v>18.845</v>
+      </c>
+      <c r="H277" s="4">
+        <f>IF(G277&gt;0,1000/G277,"")</f>
+        <v/>
+      </c>
+      <c r="I277" s="3" t="n">
+        <v>18.045</v>
+      </c>
+      <c r="J277" s="3" t="n">
+        <v>18.025</v>
+      </c>
+      <c r="K277" s="3" t="n">
+        <v>3.206</v>
+      </c>
+      <c r="L277" s="3" t="n">
+        <v>4.082</v>
+      </c>
+      <c r="M277" s="3" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="N277" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="O277" s="2" t="inlineStr">
+        <is>
+          <t>masque30c_B0, masque30c_B1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14373,7 +16565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q37"/>
+  <dimension ref="A1:Y37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -14393,6 +16585,14 @@
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14488,6 +16688,46 @@
           <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
         </is>
       </c>
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="S2" s="1" t="inlineStr">
+        <is>
+          <t>9b. Eau au sol a 10 %</t>
+        </is>
+      </c>
+      <c r="T2" s="1" t="inlineStr">
+        <is>
+          <t>9e. Essai : creux en trilineaire (abandonne)</t>
+        </is>
+      </c>
+      <c r="U2" s="1" t="inlineStr">
+        <is>
+          <t>10a. Reflet seulement dans l'eau (masque par blocs), eau 0,1</t>
+        </is>
+      </c>
+      <c r="V2" s="1" t="inlineStr">
+        <is>
+          <t>10b. Reflet seulement dans l'eau, eau 0,3</t>
+        </is>
+      </c>
+      <c r="W2" s="1" t="inlineStr">
+        <is>
+          <t>10c. Reflet seulement dans l'eau, eau 1</t>
+        </is>
+      </c>
+      <c r="X2" s="1" t="inlineStr">
+        <is>
+          <t>10e1. Essai masque : 1 point par pixel du miroir (creux manques)</t>
+        </is>
+      </c>
+      <c r="Y2" s="1" t="inlineStr">
+        <is>
+          <t>10e3. Essai masque : faisceaux seulement dans les flaques (pores plus sombres)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -14559,6 +16799,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y3" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A3,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -14630,6 +16902,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y4" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A4,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -14701,6 +17005,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y5" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A5,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -14772,6 +17108,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y6" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A6,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -14843,6 +17211,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y7" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A7,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -14914,6 +17314,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y8" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A8,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -14985,6 +17417,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y9" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A9,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -15056,6 +17520,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y10" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A10,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -15127,6 +17623,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y11" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A11,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -15198,6 +17726,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y12" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A12,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -15269,6 +17829,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y13" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A13,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -15340,6 +17932,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y14" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A14,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -15411,6 +18035,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y15" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A15,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -15482,6 +18138,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y16" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A16,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -15553,6 +18241,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y17" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A17,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -15624,6 +18344,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,Q$2),"")</f>
         <v/>
       </c>
+      <c r="R18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,R$2),"")</f>
+        <v/>
+      </c>
+      <c r="S18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,S$2),"")</f>
+        <v/>
+      </c>
+      <c r="T18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,T$2),"")</f>
+        <v/>
+      </c>
+      <c r="U18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,U$2),"")</f>
+        <v/>
+      </c>
+      <c r="V18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,V$2),"")</f>
+        <v/>
+      </c>
+      <c r="W18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,W$2),"")</f>
+        <v/>
+      </c>
+      <c r="X18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,X$2),"")</f>
+        <v/>
+      </c>
+      <c r="Y18" s="4">
+        <f>IFERROR(AVERAGEIFS(Mesures!$H:$H,Mesures!$F:$F,$A18,Mesures!$C:$C,Y$2),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -15718,6 +18470,46 @@
           <t>8. Longueur exacte des faisceaux arretes par le sol (bout des taches rasantes)</t>
         </is>
       </c>
+      <c r="R21" s="1" t="inlineStr">
+        <is>
+          <t>9a. Eau au sol : creux, flaques nettes, variante seche du shader</t>
+        </is>
+      </c>
+      <c r="S21" s="1" t="inlineStr">
+        <is>
+          <t>9b. Eau au sol a 10 %</t>
+        </is>
+      </c>
+      <c r="T21" s="1" t="inlineStr">
+        <is>
+          <t>9e. Essai : creux en trilineaire (abandonne)</t>
+        </is>
+      </c>
+      <c r="U21" s="1" t="inlineStr">
+        <is>
+          <t>10a. Reflet seulement dans l'eau (masque par blocs), eau 0,1</t>
+        </is>
+      </c>
+      <c r="V21" s="1" t="inlineStr">
+        <is>
+          <t>10b. Reflet seulement dans l'eau, eau 0,3</t>
+        </is>
+      </c>
+      <c r="W21" s="1" t="inlineStr">
+        <is>
+          <t>10c. Reflet seulement dans l'eau, eau 1</t>
+        </is>
+      </c>
+      <c r="X21" s="1" t="inlineStr">
+        <is>
+          <t>10e1. Essai masque : 1 point par pixel du miroir (creux manques)</t>
+        </is>
+      </c>
+      <c r="Y21" s="1" t="inlineStr">
+        <is>
+          <t>10e3. Essai masque : faisceaux seulement dans les flaques (pores plus sombres)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -15789,6 +18581,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y22" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A22,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -15860,6 +18684,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y23" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A23,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -15931,6 +18787,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y24" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A24,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -16002,6 +18890,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y25" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A25,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -16073,6 +18993,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y26" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A26,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -16144,6 +19096,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y27" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A27,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -16215,6 +19199,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y28" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A28,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -16286,6 +19302,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y29" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A29,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -16357,6 +19405,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y30" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A30,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -16428,6 +19508,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y31" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A31,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -16499,6 +19611,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y32" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A32,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -16570,6 +19714,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y33" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A33,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -16641,6 +19817,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y34" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A34,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -16712,6 +19920,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y35" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A35,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -16783,6 +20023,38 @@
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,Q$21),"")</f>
         <v/>
       </c>
+      <c r="R36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y36" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A36,Mesures!$C:$C,Y$21),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -16852,6 +20124,38 @@
       </c>
       <c r="Q37" s="3">
         <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,Q$21),"")</f>
+        <v/>
+      </c>
+      <c r="R37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,R$21),"")</f>
+        <v/>
+      </c>
+      <c r="S37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,S$21),"")</f>
+        <v/>
+      </c>
+      <c r="T37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,T$21),"")</f>
+        <v/>
+      </c>
+      <c r="U37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,U$21),"")</f>
+        <v/>
+      </c>
+      <c r="V37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,V$21),"")</f>
+        <v/>
+      </c>
+      <c r="W37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,W$21),"")</f>
+        <v/>
+      </c>
+      <c r="X37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,X$21),"")</f>
+        <v/>
+      </c>
+      <c r="Y37" s="3">
+        <f>IFERROR(AVERAGEIFS(Mesures!$I:$I,Mesures!$F:$F,$A37,Mesures!$C:$C,Y$21),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>